<commit_message>
Anomalies SF2-RMCP — 25/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF2-RMCP/anomalies.xlsx
+++ b/presentation/SF2-RMCP/anomalies.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -66,11 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -456,9 +460,10 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,17 +554,823 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>Nb anomalies</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>Anomalie</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Action recommandée</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>13377364</v>
+      </c>
+      <c r="B2" t="n">
+        <v>4002487243</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ronde inspection 7j Ensacheuse</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>OR004002487243</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-002506</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LIGNE ENSACHAGE PRODUIT FINIT</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>S-PC-2506</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>IP1020260810</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>13736894</v>
+      </c>
+      <c r="B3" t="n">
+        <v>4002815776</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Contrôle fermeture brûleur</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>OR004002815776</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-COMBUS-001501-SURV-ZS4706</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FIN DE COURSE DE FERMETURE BRULEUR</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S-PC-ZS4706</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>13736896</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4002815778</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ENTRETIEN SALLE TECHNIQUE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>OR004002815778</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SF02-FM-BATI-SLTECH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SALLE TECHNIQUE ATELIER MCP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>13736844</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4002815792</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Contrôle détecteur flamme XY</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>OR004002815792</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-COMBUS-001501-SURV-XY4705</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DETECTEUR DE FLAMME DU BRULEUR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S-PC-YX4705</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>13736845</v>
+      </c>
+      <c r="B6" t="n">
+        <v>4002815793</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PEVENTIF 7j DCS CAC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>OR004002815793</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-COMBUS-001501-ARAU</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ARMOIRE AUTOMATE CHAMBRE MCP</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>S-PC-API-C-MCP</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>13736910</v>
+      </c>
+      <c r="B7" t="n">
+        <v>4002815798</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Contrôle dosometre phosphate</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>OR004002815798</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-PRPULP-WT1801</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>DOSOMETRE DE LA CHAUX</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>S-PC-WT1801</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>13736885</v>
+      </c>
+      <c r="B8" t="n">
+        <v>4002815806</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ronde inspection 7j DCS</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>OR004002815806</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SF02-FM-BATI-SLTECH-DCSMCP</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SYSTÈME NUMÉRIQUE CONTRÔLE ET COMMANDE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>S-PC-MCP-DCS</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>13736878</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4002815820</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PREVENTIF SYSTEMATIQUE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>OR004002815820</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-CICHAU-02301A-SURV-KV2301A4</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ELECTROVANNE FLUIDISATION SILO 2301A</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>S-PC-KV2301A-4</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>13736900</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4002815822</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PEVENTIF 7J INSTRUM CAC</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>OR004002815822</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SF02-FM-0MCP-COMBUS-001501-SURV</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CONTRÔLE ET SURVEILLANCE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NOUVEAU PT_SAP</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SF2-RMCP</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>GM8</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>IP1020260921</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>

</xml_diff>